<commit_message>
Small change to guidance on ACM-24
</commit_message>
<xml_diff>
--- a/AIRBDS Core Metric scoring v0.3 - _initials_-_#_ TEMPLATE.xlsx
+++ b/AIRBDS Core Metric scoring v0.3 - _initials_-_#_ TEMPLATE.xlsx
@@ -7,7 +7,9 @@
     <sheet state="visible" name="Scoring" sheetId="2" r:id="rId6"/>
     <sheet state="visible" name="Lookups" sheetId="3" r:id="rId7"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">Scoring!$A$1:$K$29</definedName>
+  </definedNames>
   <calcPr/>
 </workbook>
 </file>
@@ -165,7 +167,7 @@
     <t>Licence</t>
   </si>
   <si>
-    <t>Is the dataset released with a clear licence or usage agreement?</t>
+    <t>Is the dataset released with a clear licence or terms of use?</t>
   </si>
   <si>
     <r>
@@ -482,7 +484,40 @@
     <t>If the dataset contains data from animal or human subjects, does the dataset include an ethical assessment that covers acquisition?</t>
   </si>
   <si>
-    <t>This includes consent, sampling methods, regulatory compliance, and funding sources. The acquisition should be described along accepted principles, like the Belmont, Menlo, or CARE principles, sufficient for its proper evaluation in context of intended use. If the dataset contains no human or animal data, mark the question "Yes".</t>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">This includes consent, sampling methods, regulatory compliance, and funding sources. The acquisition should be described using an appropriate framework, like the Belmont, </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>Menlo</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve">, or </t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+        <color rgb="FF1155CC"/>
+        <u/>
+      </rPr>
+      <t>CARE</t>
+    </r>
+    <r>
+      <rPr>
+        <rFont val="Arial"/>
+      </rPr>
+      <t xml:space="preserve"> principles, sufficient for its proper evaluation in context of intended use. If the dataset contains no human or animal data, mark the question "Yes".</t>
+    </r>
   </si>
   <si>
     <t>ACM-25</t>
@@ -1060,6 +1095,7 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:K29" displayName="Table1" name="Table1" id="1">
+  <autoFilter ref="$A$1:$K$29"/>
   <tableColumns count="11">
     <tableColumn name="Q ID" id="1"/>
     <tableColumn name="Mapped from" id="2"/>
@@ -5368,7 +5404,7 @@
       <c r="F25" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="G25" s="23" t="s">
+      <c r="G25" s="28" t="s">
         <v>143</v>
       </c>
       <c r="H25" s="24" t="s">
@@ -10410,10 +10446,11 @@
     <hyperlink r:id="rId1" location=":~:text=Molecular%20Data%20Usage,the%20molecular%20databases." ref="G5"/>
     <hyperlink r:id="rId2" location=":~:text=have%20these%20certified.-,FAIR%20Principles,-FAIR%20Principles%20definition" ref="G7"/>
     <hyperlink r:id="rId3" ref="B10"/>
+    <hyperlink r:id="rId4" ref="G25"/>
   </hyperlinks>
-  <drawing r:id="rId4"/>
+  <drawing r:id="rId5"/>
   <tableParts count="1">
-    <tablePart r:id="rId6"/>
+    <tablePart r:id="rId7"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>